<commit_message>
feat: simplify bulk catalog template
</commit_message>
<xml_diff>
--- a/public/plantilla-catalogo-hierroexpress.xlsx
+++ b/public/plantilla-catalogo-hierroexpress.xlsx
@@ -6,8 +6,6 @@
     <sheet name="INSTRUCCIONES" sheetId="1" r:id="rId1"/>
     <sheet name="CATEGORIAS" sheetId="2" r:id="rId2"/>
     <sheet name="PRODUCTOS" sheetId="3" r:id="rId3"/>
-    <sheet name="ATRIBUTOS" sheetId="4" r:id="rId4"/>
-    <sheet name="Subcategorias" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -401,188 +399,180 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:B5"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="105.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="110.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Carga masiva de productos</v>
+        <v>Paso</v>
       </c>
       <c r="B1" t="str">
-        <v>CATEGORIAS</v>
-      </c>
-      <c r="C1" t="str">
-        <v>PRODUCTOS</v>
-      </c>
-      <c r="D1" t="str">
-        <v>ATRIBUTOS</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Subcategorias</v>
+        <v>Detalle</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Complete las hojas CATEGORIAS y PRODUCTOS. No cambie los nombres de columnas.</v>
+        <v>1. Categorías</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Escriba los nombres de categorías y subcategorías. No use IDs ni códigos.</v>
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="str">
+        <v>2. Productos</v>
+      </c>
       <c r="B3" t="str">
-        <v>id y name son obligatorios. parentCategoryId es opcional.</v>
+        <v>Complete una fila por producto. En Categoría y Subcategoría escriba exactamente los nombres usados en la primera hoja.</v>
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="str">
-        <v>NAME, PRICE y CategoryID son los campos principales. Los productos con el mismo nombre no se duplican.</v>
+      <c r="A4" t="str">
+        <v>3. Atributos</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Opcional: indique, por ejemplo, Medida y 20 x 20 mm. El sistema los crea automáticamente.</v>
       </c>
     </row>
     <row r="5">
-      <c r="D5" t="str">
-        <v>Opcional. Id, Name y Units1. Después puede asignarlos en PRODUCTOS mediante at1Id a at4Id.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="E6" t="str">
-        <v>Opcional. La columna B es el nombre y D el id de la categoría principal.</v>
+      <c r="A5" t="str">
+        <v>Importante</v>
+      </c>
+      <c r="B5" t="str">
+        <v>No cambie los nombres de las columnas. Puede eliminar las filas de ejemplo antes de importar.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:B3"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="36.83203125" customWidth="1"/>
+    <col min="2" max="2" width="36.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>id</v>
+        <v>Categoría</v>
       </c>
       <c r="B1" t="str">
-        <v>name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>icon</v>
-      </c>
-      <c r="D1" t="str">
-        <v>parentCategoryId</v>
+        <v>Subcategoría</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" t="str">
+        <v>Caños</v>
       </c>
       <c r="B2" t="str">
-        <v>CAÑOS</v>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v/>
+        <v>Cuadrados</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>2</v>
+      <c r="A3" t="str">
+        <v>Vigas</v>
       </c>
       <c r="B3" t="str">
-        <v>VIGAS</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Caño cuadrado</v>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4">
-        <v>1</v>
+        <v>IPN</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:S3"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="42.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="34.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="22.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>NAME</v>
+        <v>Producto</v>
       </c>
       <c r="B1" t="str">
-        <v>PRICE</v>
+        <v>Precio USD</v>
       </c>
       <c r="C1" t="str">
-        <v>Image</v>
+        <v>Imagen</v>
       </c>
       <c r="D1" t="str">
-        <v>CategoryID</v>
+        <v>Categoría</v>
       </c>
       <c r="E1" t="str">
-        <v>at1Id</v>
+        <v>Subcategoría</v>
       </c>
       <c r="F1" t="str">
-        <v>valor</v>
+        <v>Descripción</v>
       </c>
       <c r="G1" t="str">
-        <v>at2Id</v>
+        <v>Stock</v>
       </c>
       <c r="H1" t="str">
-        <v>valor.1</v>
+        <v>Atributo 1</v>
       </c>
       <c r="I1" t="str">
-        <v>at3Id</v>
+        <v>Valor 1</v>
       </c>
       <c r="J1" t="str">
-        <v>valor.2</v>
+        <v>Unidad 1</v>
       </c>
       <c r="K1" t="str">
-        <v>at4Id</v>
+        <v>Atributo 2</v>
       </c>
       <c r="L1" t="str">
-        <v>valor.3</v>
+        <v>Valor 2</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Unidad 2</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Atributo 3</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Valor 3</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Unidad 3</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Atributo 4</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Valor 4</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Unidad 4</v>
       </c>
     </row>
     <row r="2">
@@ -595,31 +585,52 @@
       <c r="C2" t="str">
         <v/>
       </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
+      <c r="D2" t="str">
+        <v>Caños</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Cuadrados</v>
       </c>
       <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Medida</v>
+      </c>
+      <c r="I2" t="str">
         <v>20 x 20 mm</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
       <c r="J2" t="str">
-        <v/>
+        <v>mm</v>
       </c>
       <c r="K2" t="str">
         <v/>
       </c>
       <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
         <v/>
       </c>
     </row>
@@ -633,134 +644,58 @@
       <c r="C3" t="str">
         <v/>
       </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
+      <c r="D3" t="str">
+        <v>Vigas</v>
+      </c>
+      <c r="E3" t="str">
+        <v>IPN</v>
       </c>
       <c r="F3" t="str">
-        <v>100 mm</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="G3">
+        <v>0</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>Altura</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>mm</v>
       </c>
       <c r="K3" t="str">
         <v/>
       </c>
       <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Units1</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Medida</v>
-      </c>
-      <c r="C2" t="str">
-        <v>mm</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>A</v>
-      </c>
-      <c r="B1" t="str">
-        <v>B</v>
-      </c>
-      <c r="C1" t="str">
-        <v>C</v>
-      </c>
-      <c r="D1" t="str">
-        <v>D</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v>Cuadrados</v>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v/>
-      </c>
-      <c r="B3" t="str">
-        <v>IPN</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>